<commit_message>
feat(map): Ozon, Wildberries and Yandex Market pickup-point layers; drop expert picks
Competitor PVZ for Tashkent city, each brand checked against its own site
(WB public point list, Ozon pickup map) and Yandex Maps chain pages.
Expert picks, consensus layer, ?pick= mode and the expert guide are removed.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/pvz_shortlist.xlsx
+++ b/data/pvz_shortlist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Места под ПВЗ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Места под ПВЗ" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Места под ПВЗ'!$A$1:$Y$183</definedName>
@@ -753,10 +753,10 @@
         <v>31.8</v>
       </c>
       <c r="U3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="V3" t="n">
-        <v>500</v>
+        <v>900</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
@@ -846,7 +846,7 @@
         <v>141</v>
       </c>
       <c r="U4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="V4" t="n">
         <v>1400</v>
@@ -939,7 +939,7 @@
         <v>28.3</v>
       </c>
       <c r="U5" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="V5" t="n">
         <v>450</v>
@@ -1032,7 +1032,7 @@
         <v>141</v>
       </c>
       <c r="U6" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="V6" t="n">
         <v>918</v>
@@ -1125,7 +1125,7 @@
         <v>122.7</v>
       </c>
       <c r="U7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V7" t="n">
         <v>150</v>
@@ -1311,10 +1311,10 @@
         <v>139.7</v>
       </c>
       <c r="U9" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="V9" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
@@ -1404,10 +1404,10 @@
         <v>139.7</v>
       </c>
       <c r="U10" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="V10" t="n">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
@@ -1497,10 +1497,10 @@
         <v>59.2</v>
       </c>
       <c r="U11" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="V11" t="n">
-        <v>500</v>
+        <v>450</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
@@ -1776,10 +1776,10 @@
         <v>98.2</v>
       </c>
       <c r="U14" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="V14" t="n">
-        <v>1300</v>
+        <v>800</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>
@@ -1869,10 +1869,10 @@
         <v>98.2</v>
       </c>
       <c r="U15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="V15" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="W15" t="inlineStr">
         <is>
@@ -1962,7 +1962,7 @@
         <v>31.8</v>
       </c>
       <c r="U16" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="V16" t="n">
         <v>500</v>
@@ -2055,7 +2055,7 @@
         <v>98.2</v>
       </c>
       <c r="U17" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="V17" t="n">
         <v>700</v>
@@ -2148,7 +2148,7 @@
         <v>48.5</v>
       </c>
       <c r="U18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V18" t="n">
         <v>1400</v>
@@ -2244,7 +2244,7 @@
         <v>17</v>
       </c>
       <c r="V19" t="n">
-        <v>600</v>
+        <v>450</v>
       </c>
       <c r="W19" t="inlineStr">
         <is>
@@ -2334,7 +2334,7 @@
         <v>59.2</v>
       </c>
       <c r="U20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V20" t="n">
         <v>200</v>
@@ -2520,7 +2520,7 @@
         <v>47.6</v>
       </c>
       <c r="U22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V22" t="n">
         <v>550</v>
@@ -2704,7 +2704,7 @@
         <v>139.7</v>
       </c>
       <c r="U24" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="V24" t="n">
         <v>700</v>
@@ -2797,7 +2797,7 @@
         <v>139.7</v>
       </c>
       <c r="U25" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="V25" t="n">
         <v>350</v>
@@ -3076,7 +3076,7 @@
         <v>141</v>
       </c>
       <c r="U28" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V28" t="n">
         <v>500</v>
@@ -3169,7 +3169,7 @@
         <v>28.3</v>
       </c>
       <c r="U29" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V29" t="n">
         <v>350</v>
@@ -3353,10 +3353,10 @@
         <v>139.7</v>
       </c>
       <c r="U31" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="V31" t="n">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="W31" t="inlineStr">
         <is>
@@ -3446,7 +3446,7 @@
         <v>139.7</v>
       </c>
       <c r="U32" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="V32" t="n">
         <v>300</v>
@@ -3723,9 +3723,11 @@
         <v>98.2</v>
       </c>
       <c r="U35" t="n">
-        <v>1</v>
-      </c>
-      <c r="V35" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="V35" t="n">
+        <v>800</v>
+      </c>
       <c r="W35" t="inlineStr">
         <is>
           <t>рекомендуемая</t>
@@ -3814,9 +3816,11 @@
         <v>98.2</v>
       </c>
       <c r="U36" t="n">
-        <v>0</v>
-      </c>
-      <c r="V36" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="V36" t="n">
+        <v>3876</v>
+      </c>
       <c r="W36" t="inlineStr">
         <is>
           <t>рекомендуемая</t>
@@ -3908,7 +3912,7 @@
         <v>16</v>
       </c>
       <c r="V37" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="W37" t="inlineStr">
         <is>
@@ -3998,7 +4002,7 @@
         <v>59.2</v>
       </c>
       <c r="U38" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="V38" t="n">
         <v>250</v>
@@ -4091,7 +4095,7 @@
         <v>122.7</v>
       </c>
       <c r="U39" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V39" t="n">
         <v>350</v>
@@ -4184,7 +4188,7 @@
         <v>47.6</v>
       </c>
       <c r="U40" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="V40" t="n">
         <v>70</v>
@@ -4461,7 +4465,7 @@
         <v>59.2</v>
       </c>
       <c r="U43" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="V43" t="n">
         <v>200</v>
@@ -4554,10 +4558,10 @@
         <v>31.8</v>
       </c>
       <c r="U44" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="V44" t="n">
-        <v>500</v>
+        <v>900</v>
       </c>
       <c r="W44" t="inlineStr">
         <is>
@@ -4647,7 +4651,7 @@
         <v>28.3</v>
       </c>
       <c r="U45" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="V45" t="n">
         <v>250</v>
@@ -4833,7 +4837,7 @@
         <v>139.7</v>
       </c>
       <c r="U47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V47" t="n">
         <v>500</v>
@@ -4926,7 +4930,7 @@
         <v>28.3</v>
       </c>
       <c r="U48" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="V48" t="n">
         <v>350</v>
@@ -5019,10 +5023,10 @@
         <v>47.6</v>
       </c>
       <c r="U49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V49" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="W49" t="inlineStr">
         <is>
@@ -5112,7 +5116,7 @@
         <v>28.3</v>
       </c>
       <c r="U50" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="V50" t="n">
         <v>450</v>
@@ -5205,10 +5209,10 @@
         <v>48.5</v>
       </c>
       <c r="U51" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="V51" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="W51" t="inlineStr">
         <is>
@@ -5298,7 +5302,7 @@
         <v>122.7</v>
       </c>
       <c r="U52" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V52" t="n">
         <v>150</v>
@@ -5391,7 +5395,7 @@
         <v>31.8</v>
       </c>
       <c r="U53" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="V53" t="n">
         <v>500</v>
@@ -5852,7 +5856,7 @@
         <v>59.2</v>
       </c>
       <c r="U58" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V58" t="n">
         <v>499</v>
@@ -5945,7 +5949,7 @@
         <v>122.7</v>
       </c>
       <c r="U59" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V59" t="n">
         <v>180</v>
@@ -6041,7 +6045,7 @@
         <v>2</v>
       </c>
       <c r="V60" t="n">
-        <v>2</v>
+        <v>450</v>
       </c>
       <c r="W60" t="inlineStr">
         <is>
@@ -6222,7 +6226,7 @@
         <v>184.9</v>
       </c>
       <c r="U62" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V62" t="n">
         <v>200</v>
@@ -6315,10 +6319,10 @@
         <v>213.9</v>
       </c>
       <c r="U63" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V63" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="W63" t="inlineStr">
         <is>
@@ -6408,10 +6412,10 @@
         <v>270.6</v>
       </c>
       <c r="U64" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V64" t="n">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="W64" t="inlineStr">
         <is>
@@ -6501,10 +6505,10 @@
         <v>270.6</v>
       </c>
       <c r="U65" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V65" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="W65" t="inlineStr">
         <is>
@@ -6964,7 +6968,7 @@
         <v>184.9</v>
       </c>
       <c r="U70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V70" t="inlineStr"/>
       <c r="W70" t="inlineStr">
@@ -7146,7 +7150,7 @@
         <v>270.6</v>
       </c>
       <c r="U72" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V72" t="n">
         <v>3500</v>
@@ -7239,7 +7243,7 @@
         <v>270.6</v>
       </c>
       <c r="U73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V73" t="inlineStr"/>
       <c r="W73" t="inlineStr">
@@ -7789,7 +7793,7 @@
         <v>213.9</v>
       </c>
       <c r="U79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V79" t="n">
         <v>1000</v>
@@ -7978,7 +7982,7 @@
         <v>1</v>
       </c>
       <c r="V81" t="n">
-        <v>1100</v>
+        <v>3000</v>
       </c>
       <c r="W81" t="inlineStr">
         <is>
@@ -8068,9 +8072,11 @@
         <v>270.6</v>
       </c>
       <c r="U82" t="n">
-        <v>0</v>
-      </c>
-      <c r="V82" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="V82" t="n">
+        <v>1200</v>
+      </c>
       <c r="W82" t="inlineStr">
         <is>
           <t>рекомендуемая</t>
@@ -8344,7 +8350,7 @@
         <v>2</v>
       </c>
       <c r="V85" t="n">
-        <v>1100</v>
+        <v>3000</v>
       </c>
       <c r="W85" t="inlineStr">
         <is>
@@ -8798,7 +8804,7 @@
         <v>184.9</v>
       </c>
       <c r="U90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V90" t="inlineStr"/>
       <c r="W90" t="inlineStr">
@@ -8889,11 +8895,9 @@
         <v>213.9</v>
       </c>
       <c r="U91" t="n">
-        <v>1</v>
-      </c>
-      <c r="V91" t="n">
-        <v>1100</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="V91" t="inlineStr"/>
       <c r="W91" t="inlineStr">
         <is>
           <t>рекомендуемая</t>
@@ -9073,7 +9077,7 @@
         <v>184.9</v>
       </c>
       <c r="U93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V93" t="inlineStr"/>
       <c r="W93" t="inlineStr">
@@ -9528,9 +9532,11 @@
         <v>270.6</v>
       </c>
       <c r="U98" t="n">
-        <v>0</v>
-      </c>
-      <c r="V98" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="V98" t="n">
+        <v>1200</v>
+      </c>
       <c r="W98" t="inlineStr">
         <is>
           <t>рекомендуемая</t>

</xml_diff>

<commit_message>
feat(zhk): sales-office and developer phones in the registry and popup
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/pvz_shortlist.xlsx
+++ b/data/pvz_shortlist.xlsx
@@ -598,7 +598,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>41.275234</v>
@@ -636,7 +636,7 @@
         <v>14985</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="N2" t="n">
         <v>57</v>
@@ -729,7 +729,7 @@
         <v>10558</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N3" t="n">
         <v>31</v>
@@ -787,19 +787,19 @@
         <v>91</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>41.302375</v>
+        <v>41.298608</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>69.289134</v>
+        <v>69.213863</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>41.302375, 69.289134</t>
+          <t>41.298608, 69.213863</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Айбек</t>
+          <t>Чарх Камалан-3 махалля</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -808,48 +808,48 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1.1</v>
+        <v>0.4</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Яшнободский район</t>
+          <t>Чиланзарский район</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>13591</v>
+        <v>17457</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="N4" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="O4" t="n">
         <v>16</v>
       </c>
       <c r="P4" t="n">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="Q4" t="n">
         <v>0.5</v>
       </c>
       <c r="R4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S4" t="n">
-        <v>448</v>
+        <v>781</v>
       </c>
       <c r="T4" t="n">
-        <v>141</v>
+        <v>28.3</v>
       </c>
       <c r="U4" t="n">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="V4" t="n">
-        <v>918</v>
+        <v>500</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -863,7 +863,7 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.302375,69.289134</t>
+          <t>https://www.google.com/maps?q=41.298608,69.213863</t>
         </is>
       </c>
     </row>
@@ -880,19 +880,19 @@
         <v>91</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>41.298608</v>
+        <v>41.302375</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>69.213863</v>
+        <v>69.289134</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>41.298608, 69.213863</t>
+          <t>41.302375, 69.289134</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Чарх Камалан-3 махалля</t>
+          <t>Айбек</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -901,48 +901,48 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>0.4</v>
+        <v>1.1</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Чиланзарский район</t>
+          <t>Яшнободский район</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>17457</v>
+        <v>13591</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N5" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="O5" t="n">
         <v>16</v>
       </c>
       <c r="P5" t="n">
-        <v>46</v>
+        <v>79</v>
       </c>
       <c r="Q5" t="n">
         <v>0.5</v>
       </c>
       <c r="R5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>781</v>
+        <v>448</v>
       </c>
       <c r="T5" t="n">
-        <v>28.3</v>
+        <v>141</v>
       </c>
       <c r="U5" t="n">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="V5" t="n">
-        <v>500</v>
+        <v>918</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -956,7 +956,7 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.298608,69.213863</t>
+          <t>https://www.google.com/maps?q=41.302375,69.289134</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
         <v>12156</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N6" t="n">
         <v>20</v>
@@ -1063,7 +1063,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>41.329729</v>
@@ -1101,7 +1101,7 @@
         <v>10538</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N7" t="n">
         <v>52</v>
@@ -1159,19 +1159,19 @@
         <v>90</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>41.204808</v>
+        <v>41.353226</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>69.199336</v>
+        <v>69.31441100000001</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>41.204808, 69.199336</t>
+          <t>41.353226, 69.314411</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Гульшанабад махалля</t>
+          <t>Атчапар-2 махалля</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1180,48 +1180,48 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Янгихаётский район</t>
+          <t>Юнусабадский район</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>8833</v>
+        <v>5180</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N8" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="O8" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="P8" t="n">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="Q8" t="n">
         <v>0.5</v>
       </c>
       <c r="R8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S8" t="n">
-        <v>13000</v>
+        <v>4200</v>
       </c>
       <c r="T8" t="n">
-        <v>122.7</v>
+        <v>139.7</v>
       </c>
       <c r="U8" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="V8" t="n">
-        <v>1400</v>
+        <v>350</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.204808,69.199336</t>
+          <t>https://www.google.com/maps?q=41.353226,69.314411</t>
         </is>
       </c>
     </row>
@@ -1252,19 +1252,19 @@
         <v>90</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>41.353226</v>
+        <v>41.204808</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>69.31441100000001</v>
+        <v>69.199336</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>41.353226, 69.314411</t>
+          <t>41.204808, 69.199336</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Атчапар-2 махалля</t>
+          <t>Гульшанабад махалля</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1273,48 +1273,48 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Юнусабадский район</t>
+          <t>Янгихаётский район</t>
         </is>
       </c>
       <c r="L9" t="n">
-        <v>5180</v>
+        <v>8833</v>
       </c>
       <c r="M9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N9" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="O9" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P9" t="n">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="Q9" t="n">
         <v>0.5</v>
       </c>
       <c r="R9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" t="n">
+        <v>13000</v>
+      </c>
+      <c r="T9" t="n">
+        <v>122.7</v>
+      </c>
+      <c r="U9" t="n">
         <v>2</v>
       </c>
-      <c r="S9" t="n">
-        <v>4200</v>
-      </c>
-      <c r="T9" t="n">
-        <v>139.7</v>
-      </c>
-      <c r="U9" t="n">
-        <v>9</v>
-      </c>
       <c r="V9" t="n">
-        <v>350</v>
+        <v>1400</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.353226,69.314411</t>
+          <t>https://www.google.com/maps?q=41.204808,69.199336</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
         <v>11740</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N10" t="n">
         <v>14</v>
@@ -1473,7 +1473,7 @@
         <v>14912</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="N11" t="n">
         <v>50</v>
@@ -1566,7 +1566,7 @@
         <v>15593</v>
       </c>
       <c r="M12" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="N12" t="n">
         <v>35</v>
@@ -1659,7 +1659,7 @@
         <v>8891</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N13" t="n">
         <v>34</v>
@@ -1714,7 +1714,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>41.309964</v>
@@ -1752,7 +1752,7 @@
         <v>9976</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N14" t="n">
         <v>31</v>
@@ -1845,10 +1845,10 @@
         <v>7882</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="N15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="O15" t="n">
         <v>21</v>
@@ -1938,7 +1938,7 @@
         <v>13228</v>
       </c>
       <c r="M16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="N16" t="n">
         <v>28</v>
@@ -1996,19 +1996,19 @@
         <v>86</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>41.337616</v>
+        <v>41.335981</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>69.32581399999999</v>
+        <v>69.321806</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>41.337616, 69.325814</t>
+          <t>41.335981, 69.321806</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Буз-1 (Черданцева)</t>
+          <t>Буюк Ипак Йули махалля</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -2028,19 +2028,19 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>5401</v>
+        <v>5082</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N17" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="O17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P17" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="Q17" t="n">
         <v>0.5</v>
@@ -2055,7 +2055,7 @@
         <v>98.2</v>
       </c>
       <c r="U17" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="V17" t="n">
         <v>500</v>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.337616,69.325814</t>
+          <t>https://www.google.com/maps?q=41.335981,69.321806</t>
         </is>
       </c>
     </row>
@@ -2089,19 +2089,19 @@
         <v>86</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>41.314123</v>
+        <v>41.365403</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>69.301356</v>
+        <v>69.393992</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>41.314123, 69.301356</t>
+          <t>41.365403, 69.393992</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Ирригатор массив</t>
+          <t>ТТЗ-4</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2110,30 +2110,30 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Мирзо Улугбекский район</t>
+          <t>Кибрайский район</t>
         </is>
       </c>
       <c r="L18" t="n">
-        <v>6403</v>
+        <v>13404</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N18" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="O18" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="P18" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="Q18" t="n">
         <v>0.5</v>
@@ -2142,16 +2142,16 @@
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>220</v>
+        <v>1200</v>
       </c>
       <c r="T18" t="n">
-        <v>98.2</v>
+        <v>213.9</v>
       </c>
       <c r="U18" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="V18" t="n">
-        <v>500</v>
+        <v>1400</v>
       </c>
       <c r="W18" t="inlineStr">
         <is>
@@ -2165,7 +2165,7 @@
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.314123,69.301356</t>
+          <t>https://www.google.com/maps?q=41.365403,69.393992</t>
         </is>
       </c>
     </row>
@@ -2182,19 +2182,19 @@
         <v>86</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>41.365403</v>
+        <v>41.314123</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>69.393992</v>
+        <v>69.301356</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>41.365403, 69.393992</t>
+          <t>41.314123, 69.301356</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>ТТЗ-4</t>
+          <t>Ирригатор массив</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2203,30 +2203,30 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Кибрайский район</t>
+          <t>Мирзо Улугбекский район</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>13404</v>
+        <v>6403</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N19" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="O19" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="P19" t="n">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="Q19" t="n">
         <v>0.5</v>
@@ -2235,16 +2235,16 @@
         <v>1</v>
       </c>
       <c r="S19" t="n">
-        <v>1200</v>
+        <v>220</v>
       </c>
       <c r="T19" t="n">
-        <v>213.9</v>
+        <v>98.2</v>
       </c>
       <c r="U19" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="V19" t="n">
-        <v>1400</v>
+        <v>500</v>
       </c>
       <c r="W19" t="inlineStr">
         <is>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.365403,69.393992</t>
+          <t>https://www.google.com/maps?q=41.314123,69.301356</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2310,7 @@
         <v>5016</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N20" t="n">
         <v>49</v>
@@ -2368,19 +2368,19 @@
         <v>85</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>41.365496</v>
+        <v>41.350681</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>69.203898</v>
+        <v>69.266822</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>41.365496, 69.203898</t>
+          <t>41.350681, 69.266822</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Бешкурган-4</t>
+          <t>Джами махалля</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2389,30 +2389,30 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Алмазарский район</t>
+          <t>Юнусабадский район</t>
         </is>
       </c>
       <c r="L21" t="n">
-        <v>12971</v>
+        <v>4950</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N21" t="n">
+        <v>58</v>
+      </c>
+      <c r="O21" t="n">
         <v>28</v>
       </c>
-      <c r="O21" t="n">
-        <v>11</v>
-      </c>
       <c r="P21" t="n">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="Q21" t="n">
         <v>0.5</v>
@@ -2421,16 +2421,16 @@
         <v>1</v>
       </c>
       <c r="S21" t="n">
-        <v>313</v>
+        <v>126</v>
       </c>
       <c r="T21" t="n">
-        <v>59.2</v>
+        <v>139.7</v>
       </c>
       <c r="U21" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="V21" t="n">
-        <v>570</v>
+        <v>450</v>
       </c>
       <c r="W21" t="inlineStr">
         <is>
@@ -2444,7 +2444,7 @@
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.365496,69.203898</t>
+          <t>https://www.google.com/maps?q=41.350681,69.266822</t>
         </is>
       </c>
     </row>
@@ -2461,19 +2461,19 @@
         <v>85</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>41.350681</v>
+        <v>41.365496</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>69.266822</v>
+        <v>69.203898</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>41.350681, 69.266822</t>
+          <t>41.365496, 69.203898</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Джами махалля</t>
+          <t>Бешкурган-4</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2482,30 +2482,30 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Юнусабадский район</t>
+          <t>Алмазарский район</t>
         </is>
       </c>
       <c r="L22" t="n">
-        <v>4950</v>
+        <v>12971</v>
       </c>
       <c r="M22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N22" t="n">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="O22" t="n">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="P22" t="n">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="Q22" t="n">
         <v>0.5</v>
@@ -2514,16 +2514,16 @@
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>126</v>
+        <v>313</v>
       </c>
       <c r="T22" t="n">
-        <v>139.7</v>
+        <v>59.2</v>
       </c>
       <c r="U22" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="V22" t="n">
-        <v>450</v>
+        <v>570</v>
       </c>
       <c r="W22" t="inlineStr">
         <is>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.350681,69.266822</t>
+          <t>https://www.google.com/maps?q=41.365496,69.203898</t>
         </is>
       </c>
     </row>
@@ -2554,19 +2554,19 @@
         <v>84</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>41.271165</v>
+        <v>41.283946</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>69.311927</v>
+        <v>69.359775</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>41.271165, 69.311927</t>
+          <t>41.283946, 69.359775</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Ок Уй махалля</t>
+          <t>Авиасозлар-1</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2575,30 +2575,30 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Мирабадский район</t>
+          <t>Яшнободский район</t>
         </is>
       </c>
       <c r="L23" t="n">
-        <v>10553</v>
+        <v>13526</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="N23" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="O23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P23" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="Q23" t="n">
         <v>0.5</v>
@@ -2607,16 +2607,16 @@
         <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>726</v>
+        <v>480</v>
       </c>
       <c r="T23" t="n">
-        <v>48.5</v>
+        <v>141</v>
       </c>
       <c r="U23" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V23" t="n">
-        <v>1400</v>
+        <v>900</v>
       </c>
       <c r="W23" t="inlineStr">
         <is>
@@ -2630,7 +2630,7 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.271165,69.311927</t>
+          <t>https://www.google.com/maps?q=41.283946,69.359775</t>
         </is>
       </c>
     </row>
@@ -2647,19 +2647,19 @@
         <v>84</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>41.32587</v>
+        <v>41.271165</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>69.31358299999999</v>
+        <v>69.311927</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>41.325870, 69.313583</t>
+          <t>41.271165, 69.311927</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Янги Алмачи махалля</t>
+          <t>Ок Уй махалля</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2668,48 +2668,48 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Мирзо Улугбекский район</t>
+          <t>Мирабадский район</t>
         </is>
       </c>
       <c r="L24" t="n">
-        <v>3115</v>
+        <v>10553</v>
       </c>
       <c r="M24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N24" t="n">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="O24" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="P24" t="n">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="Q24" t="n">
         <v>0.5</v>
       </c>
       <c r="R24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S24" t="n">
-        <v>759</v>
+        <v>726</v>
       </c>
       <c r="T24" t="n">
-        <v>98.2</v>
+        <v>48.5</v>
       </c>
       <c r="U24" t="n">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="V24" t="n">
-        <v>500</v>
+        <v>1400</v>
       </c>
       <c r="W24" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.325870,69.313583</t>
+          <t>https://www.google.com/maps?q=41.271165,69.311927</t>
         </is>
       </c>
     </row>
@@ -2740,19 +2740,19 @@
         <v>84</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>41.283946</v>
+        <v>41.311064</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>69.359775</v>
+        <v>69.186525</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>41.283946, 69.359775</t>
+          <t>41.311064, 69.186525</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Авиасозлар-1</t>
+          <t>Пахтакор махалля</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2768,41 +2768,41 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Яшнободский район</t>
+          <t>Учтепинский район</t>
         </is>
       </c>
       <c r="L25" t="n">
-        <v>13526</v>
+        <v>3023</v>
       </c>
       <c r="M25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N25" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="O25" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="P25" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q25" t="n">
         <v>0.5</v>
       </c>
       <c r="R25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S25" t="n">
-        <v>480</v>
+        <v>1777</v>
       </c>
       <c r="T25" t="n">
-        <v>141</v>
+        <v>47.6</v>
       </c>
       <c r="U25" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="V25" t="n">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="W25" t="inlineStr">
         <is>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.283946,69.359775</t>
+          <t>https://www.google.com/maps?q=41.311064,69.186525</t>
         </is>
       </c>
     </row>
@@ -2830,22 +2830,22 @@
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>41.311064</v>
+        <v>41.31798</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>69.186525</v>
+        <v>69.27772899999999</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>41.311064, 69.186525</t>
+          <t>41.317980, 69.277729</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Пахтакор махалля</t>
+          <t>Кашгар (Ц-4)</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2854,48 +2854,48 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Учтепинский район</t>
+          <t>Юнусабадский район</t>
         </is>
       </c>
       <c r="L26" t="n">
-        <v>3023</v>
+        <v>6739</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N26" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O26" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="P26" t="n">
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="Q26" t="n">
         <v>0.5</v>
       </c>
       <c r="R26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>1777</v>
+        <v>0</v>
       </c>
       <c r="T26" t="n">
-        <v>47.6</v>
+        <v>139.7</v>
       </c>
       <c r="U26" t="n">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="V26" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="W26" t="inlineStr">
         <is>
@@ -2909,7 +2909,7 @@
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.311064,69.186525</t>
+          <t>https://www.google.com/maps?q=41.317980,69.277729</t>
         </is>
       </c>
     </row>
@@ -2926,19 +2926,19 @@
         <v>83</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>41.31798</v>
+        <v>41.24277</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>69.27772899999999</v>
+        <v>69.36640199999999</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>41.317980, 69.277729</t>
+          <t>41.242770, 69.366402</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Кашгар (Ц-4)</t>
+          <t>Абай махалля</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2947,49 +2947,47 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Юнусабадский район</t>
+          <t>Бектемирский район</t>
         </is>
       </c>
       <c r="L27" t="n">
-        <v>6739</v>
+        <v>8381</v>
       </c>
       <c r="M27" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N27" t="n">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="O27" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="P27" t="n">
-        <v>95</v>
+        <v>10</v>
       </c>
       <c r="Q27" t="n">
         <v>0.5</v>
       </c>
       <c r="R27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S27" t="n">
-        <v>0</v>
+        <v>828</v>
       </c>
       <c r="T27" t="n">
-        <v>139.7</v>
+        <v>60.2</v>
       </c>
       <c r="U27" t="n">
-        <v>58</v>
-      </c>
-      <c r="V27" t="n">
-        <v>700</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr">
         <is>
           <t>рекомендуемая</t>
@@ -3002,7 +3000,7 @@
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.317980,69.277729</t>
+          <t>https://www.google.com/maps?q=41.242770,69.366402</t>
         </is>
       </c>
     </row>
@@ -3054,7 +3052,7 @@
         <v>7101</v>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N28" t="n">
         <v>15</v>
@@ -3112,19 +3110,19 @@
         <v>82</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>41.296436</v>
+        <v>41.322155</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>69.332471</v>
+        <v>69.3293</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>41.296436, 69.332471</t>
+          <t>41.322155, 69.329300</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Куксарай махалля</t>
+          <t>Алмачи махалля</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3133,30 +3131,30 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Яшнободский район</t>
+          <t>Мирзо Улугбекский район</t>
         </is>
       </c>
       <c r="L29" t="n">
-        <v>4067</v>
+        <v>8916</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N29" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="O29" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="P29" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="Q29" t="n">
         <v>0.5</v>
@@ -3165,13 +3163,13 @@
         <v>1</v>
       </c>
       <c r="S29" t="n">
-        <v>488</v>
+        <v>80</v>
       </c>
       <c r="T29" t="n">
-        <v>141</v>
+        <v>98.2</v>
       </c>
       <c r="U29" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="V29" t="n">
         <v>500</v>
@@ -3188,7 +3186,7 @@
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.296436,69.332471</t>
+          <t>https://www.google.com/maps?q=41.322155,69.329300</t>
         </is>
       </c>
     </row>
@@ -3205,19 +3203,19 @@
         <v>82</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>41.370618</v>
+        <v>41.296436</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>69.29909600000001</v>
+        <v>69.332471</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>41.370618, 69.299096</t>
+          <t>41.296436, 69.332471</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Юнусабад 13-й квартал</t>
+          <t>Куксарай махалля</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3226,48 +3224,48 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Юнусабадский район</t>
+          <t>Яшнободский район</t>
         </is>
       </c>
       <c r="L30" t="n">
-        <v>22705</v>
+        <v>4067</v>
       </c>
       <c r="M30" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N30" t="n">
+        <v>25</v>
+      </c>
+      <c r="O30" t="n">
+        <v>14</v>
+      </c>
+      <c r="P30" t="n">
         <v>33</v>
-      </c>
-      <c r="O30" t="n">
-        <v>13</v>
-      </c>
-      <c r="P30" t="n">
-        <v>31</v>
       </c>
       <c r="Q30" t="n">
         <v>0.5</v>
       </c>
       <c r="R30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S30" t="n">
-        <v>0</v>
+        <v>488</v>
       </c>
       <c r="T30" t="n">
-        <v>139.7</v>
+        <v>141</v>
       </c>
       <c r="U30" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="V30" t="n">
-        <v>350</v>
+        <v>500</v>
       </c>
       <c r="W30" t="inlineStr">
         <is>
@@ -3281,7 +3279,7 @@
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.370618,69.299096</t>
+          <t>https://www.google.com/maps?q=41.296436,69.332471</t>
         </is>
       </c>
     </row>
@@ -3298,19 +3296,19 @@
         <v>82</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>41.24277</v>
+        <v>41.343199</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>69.36640199999999</v>
+        <v>69.207222</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>41.242770, 69.366402</t>
+          <t>41.343199, 69.207222</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Абай махалля</t>
+          <t>массив Ниязова</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3319,30 +3317,30 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Бектемирский район</t>
+          <t>Алмазарский район</t>
         </is>
       </c>
       <c r="L31" t="n">
-        <v>8381</v>
+        <v>6689</v>
       </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="N31" t="n">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="O31" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="P31" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="Q31" t="n">
         <v>0.5</v>
@@ -3351,15 +3349,17 @@
         <v>1</v>
       </c>
       <c r="S31" t="n">
-        <v>828</v>
+        <v>96</v>
       </c>
       <c r="T31" t="n">
-        <v>60.2</v>
+        <v>59.2</v>
       </c>
       <c r="U31" t="n">
-        <v>0</v>
-      </c>
-      <c r="V31" t="inlineStr"/>
+        <v>17</v>
+      </c>
+      <c r="V31" t="n">
+        <v>500</v>
+      </c>
       <c r="W31" t="inlineStr">
         <is>
           <t>рекомендуемая</t>
@@ -3372,7 +3372,7 @@
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.242770,69.366402</t>
+          <t>https://www.google.com/maps?q=41.343199,69.207222</t>
         </is>
       </c>
     </row>
@@ -3389,19 +3389,19 @@
         <v>82</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>41.343199</v>
+        <v>41.370618</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>69.207222</v>
+        <v>69.29909600000001</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>41.343199, 69.207222</t>
+          <t>41.370618, 69.299096</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>массив Ниязова</t>
+          <t>Юнусабад 13-й квартал</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3417,41 +3417,41 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Алмазарский район</t>
+          <t>Юнусабадский район</t>
         </is>
       </c>
       <c r="L32" t="n">
-        <v>6689</v>
+        <v>22705</v>
       </c>
       <c r="M32" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N32" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="O32" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="P32" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="Q32" t="n">
         <v>0.5</v>
       </c>
       <c r="R32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="T32" t="n">
-        <v>59.2</v>
+        <v>139.7</v>
       </c>
       <c r="U32" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="V32" t="n">
-        <v>500</v>
+        <v>350</v>
       </c>
       <c r="W32" t="inlineStr">
         <is>
@@ -3465,7 +3465,7 @@
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.343199,69.207222</t>
+          <t>https://www.google.com/maps?q=41.370618,69.299096</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
         <v>5652</v>
       </c>
       <c r="M33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N33" t="n">
         <v>49</v>
@@ -3575,19 +3575,19 @@
         <v>79</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>41.318137</v>
+        <v>41.260613</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>69.360837</v>
+        <v>69.327422</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>41.318137, 69.360837</t>
+          <t>41.260613, 69.327422</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Гульзарабад махалля</t>
+          <t>Бунёдкор махалля</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -3607,28 +3607,28 @@
         </is>
       </c>
       <c r="L34" t="n">
-        <v>7413</v>
+        <v>3292</v>
       </c>
       <c r="M34" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N34" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="O34" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="P34" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="Q34" t="n">
         <v>0.5</v>
       </c>
       <c r="R34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S34" t="n">
-        <v>0</v>
+        <v>380</v>
       </c>
       <c r="T34" t="n">
         <v>141</v>
@@ -3637,7 +3637,7 @@
         <v>3</v>
       </c>
       <c r="V34" t="n">
-        <v>650</v>
+        <v>1400</v>
       </c>
       <c r="W34" t="inlineStr">
         <is>
@@ -3651,7 +3651,7 @@
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.318137,69.360837</t>
+          <t>https://www.google.com/maps?q=41.260613,69.327422</t>
         </is>
       </c>
     </row>
@@ -3668,19 +3668,19 @@
         <v>79</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>41.260613</v>
+        <v>41.318137</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>69.327422</v>
+        <v>69.360837</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>41.260613, 69.327422</t>
+          <t>41.318137, 69.360837</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Бунёдкор махалля</t>
+          <t>Гульзарабад махалля</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3700,28 +3700,28 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>3292</v>
+        <v>7413</v>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N35" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="O35" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="P35" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="Q35" t="n">
         <v>0.5</v>
       </c>
       <c r="R35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>380</v>
+        <v>0</v>
       </c>
       <c r="T35" t="n">
         <v>141</v>
@@ -3730,7 +3730,7 @@
         <v>3</v>
       </c>
       <c r="V35" t="n">
-        <v>1400</v>
+        <v>650</v>
       </c>
       <c r="W35" t="inlineStr">
         <is>
@@ -3744,7 +3744,7 @@
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.260613,69.327422</t>
+          <t>https://www.google.com/maps?q=41.318137,69.360837</t>
         </is>
       </c>
     </row>
@@ -3796,7 +3796,7 @@
         <v>8693</v>
       </c>
       <c r="M36" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N36" t="n">
         <v>24</v>
@@ -3889,10 +3889,10 @@
         <v>2020</v>
       </c>
       <c r="M37" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N37" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="O37" t="n">
         <v>6</v>
@@ -3982,7 +3982,7 @@
         <v>9262</v>
       </c>
       <c r="M38" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N38" t="n">
         <v>19</v>
@@ -4075,7 +4075,7 @@
         <v>7484</v>
       </c>
       <c r="M39" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N39" t="n">
         <v>18</v>
@@ -4168,7 +4168,7 @@
         <v>10288</v>
       </c>
       <c r="M40" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="N40" t="n">
         <v>52</v>
@@ -4261,7 +4261,7 @@
         <v>16603</v>
       </c>
       <c r="M41" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="N41" t="n">
         <v>60</v>
@@ -4354,7 +4354,7 @@
         <v>5737</v>
       </c>
       <c r="M42" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N42" t="n">
         <v>23</v>
@@ -4447,7 +4447,7 @@
         <v>10881</v>
       </c>
       <c r="M43" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N43" t="n">
         <v>23</v>
@@ -4502,22 +4502,22 @@
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>41.323641</v>
+        <v>41.250058</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>69.341219</v>
+        <v>69.342911</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>41.323641, 69.341219</t>
+          <t>41.250058, 69.342911</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Катта Алтынтепа махалля</t>
+          <t>Аханграбо (Панельный)</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4526,30 +4526,30 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="J44" t="n">
         <v>0</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Мирзо Улугбекский район</t>
+          <t>Яшнободский район</t>
         </is>
       </c>
       <c r="L44" t="n">
-        <v>6442</v>
+        <v>4446</v>
       </c>
       <c r="M44" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N44" t="n">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="O44" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="P44" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="Q44" t="n">
         <v>0.5</v>
@@ -4561,14 +4561,12 @@
         <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>98.2</v>
+        <v>141</v>
       </c>
       <c r="U44" t="n">
-        <v>23</v>
-      </c>
-      <c r="V44" t="n">
-        <v>500</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="V44" t="inlineStr"/>
       <c r="W44" t="inlineStr">
         <is>
           <t>рекомендуемая</t>
@@ -4581,7 +4579,7 @@
       </c>
       <c r="Y44" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.323641,69.341219</t>
+          <t>https://www.google.com/maps?q=41.250058,69.342911</t>
         </is>
       </c>
     </row>
@@ -4598,19 +4596,19 @@
         <v>75</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>41.250058</v>
+        <v>41.343858</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>69.342911</v>
+        <v>69.357677</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>41.250058, 69.342911</t>
+          <t>41.343858, 69.357677</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Аханграбо (Панельный)</t>
+          <t>Буз-2 (Черданцева)</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -4619,30 +4617,30 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Яшнободский район</t>
+          <t>Мирзо Улугбекский район</t>
         </is>
       </c>
       <c r="L45" t="n">
-        <v>4446</v>
+        <v>5378</v>
       </c>
       <c r="M45" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="N45" t="n">
+        <v>35</v>
+      </c>
+      <c r="O45" t="n">
         <v>16</v>
       </c>
-      <c r="O45" t="n">
-        <v>7</v>
-      </c>
       <c r="P45" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="Q45" t="n">
         <v>0.5</v>
@@ -4654,12 +4652,14 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>141</v>
+        <v>98.2</v>
       </c>
       <c r="U45" t="n">
-        <v>0</v>
-      </c>
-      <c r="V45" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="V45" t="n">
+        <v>10</v>
+      </c>
       <c r="W45" t="inlineStr">
         <is>
           <t>рекомендуемая</t>
@@ -4672,7 +4672,7 @@
       </c>
       <c r="Y45" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.250058,69.342911</t>
+          <t>https://www.google.com/maps?q=41.343858,69.357677</t>
         </is>
       </c>
     </row>
@@ -4689,19 +4689,19 @@
         <v>75</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>41.343858</v>
+        <v>41.332115</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>69.357677</v>
+        <v>69.345438</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>41.343858, 69.357677</t>
+          <t>41.332115, 69.345438</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Буз-2 (Черданцева)</t>
+          <t>Академгородок</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -4721,19 +4721,19 @@
         </is>
       </c>
       <c r="L46" t="n">
-        <v>5378</v>
+        <v>4353</v>
       </c>
       <c r="M46" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N46" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O46" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P46" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="Q46" t="n">
         <v>0.5</v>
@@ -4748,7 +4748,7 @@
         <v>98.2</v>
       </c>
       <c r="U46" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="V46" t="n">
         <v>10</v>
@@ -4765,7 +4765,7 @@
       </c>
       <c r="Y46" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.343858,69.357677</t>
+          <t>https://www.google.com/maps?q=41.332115,69.345438</t>
         </is>
       </c>
     </row>
@@ -4817,7 +4817,7 @@
         <v>11879</v>
       </c>
       <c r="M47" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N47" t="n">
         <v>48</v>
@@ -4910,7 +4910,7 @@
         <v>10654</v>
       </c>
       <c r="M48" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="N48" t="n">
         <v>36</v>
@@ -5003,7 +5003,7 @@
         <v>12235</v>
       </c>
       <c r="M49" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N49" t="n">
         <v>46</v>
@@ -5096,7 +5096,7 @@
         <v>2530</v>
       </c>
       <c r="M50" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N50" t="n">
         <v>21</v>
@@ -5151,7 +5151,7 @@
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D51" s="2" t="n">
         <v>41.271397</v>
@@ -5189,10 +5189,10 @@
         <v>10663</v>
       </c>
       <c r="M51" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="N51" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O51" t="n">
         <v>18</v>
@@ -5247,19 +5247,19 @@
         <v>72</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>41.376688</v>
+        <v>41.265528</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>69.24778499999999</v>
+        <v>69.149665</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>41.376688, 69.247785</t>
+          <t>41.265528, 69.149665</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Ибрагим-Ата махалля</t>
+          <t>Чиланзар-31</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -5268,30 +5268,30 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Юнусабадский район</t>
+          <t>Учтепинский район</t>
         </is>
       </c>
       <c r="L52" t="n">
-        <v>2816</v>
+        <v>10778</v>
       </c>
       <c r="M52" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="N52" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="O52" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P52" t="n">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="Q52" t="n">
         <v>0.5</v>
@@ -5303,13 +5303,13 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>139.7</v>
+        <v>47.6</v>
       </c>
       <c r="U52" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="V52" t="n">
-        <v>500</v>
+        <v>2</v>
       </c>
       <c r="W52" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
       </c>
       <c r="Y52" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.376688,69.247785</t>
+          <t>https://www.google.com/maps?q=41.265528,69.149665</t>
         </is>
       </c>
     </row>
@@ -5375,10 +5375,10 @@
         <v>8748</v>
       </c>
       <c r="M53" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N53" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="O53" t="n">
         <v>17</v>
@@ -5433,19 +5433,19 @@
         <v>72</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>41.265528</v>
+        <v>41.376688</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>69.149665</v>
+        <v>69.24778499999999</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>41.265528, 69.149665</t>
+          <t>41.376688, 69.247785</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Чиланзар-31</t>
+          <t>Ибрагим-Ата махалля</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -5454,30 +5454,30 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
       <c r="J54" t="n">
         <v>0</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Учтепинский район</t>
+          <t>Юнусабадский район</t>
         </is>
       </c>
       <c r="L54" t="n">
-        <v>10778</v>
+        <v>2816</v>
       </c>
       <c r="M54" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N54" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="O54" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="P54" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="Q54" t="n">
         <v>0.5</v>
@@ -5489,13 +5489,13 @@
         <v>0</v>
       </c>
       <c r="T54" t="n">
-        <v>47.6</v>
+        <v>139.7</v>
       </c>
       <c r="U54" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="V54" t="n">
-        <v>2</v>
+        <v>500</v>
       </c>
       <c r="W54" t="inlineStr">
         <is>
@@ -5509,7 +5509,7 @@
       </c>
       <c r="Y54" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.265528,69.149665</t>
+          <t>https://www.google.com/maps?q=41.376688,69.247785</t>
         </is>
       </c>
     </row>
@@ -5614,7 +5614,7 @@
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D56" s="2" t="n">
         <v>41.283644</v>
@@ -5652,7 +5652,7 @@
         <v>5986</v>
       </c>
       <c r="M56" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N56" t="n">
         <v>33</v>
@@ -5745,10 +5745,10 @@
         <v>11138</v>
       </c>
       <c r="M57" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N57" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O57" t="n">
         <v>12</v>
@@ -5800,54 +5800,54 @@
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>41.390081</v>
+        <v>41.254507</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>69.26402400000001</v>
+        <v>69.37862699999999</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>41.390081, 69.264024</t>
+          <t>41.254507, 69.378627</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Дустамабад</t>
+          <t>Сувсоз-2 (Водник)</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>посёлок</t>
+          <t>махалля</t>
         </is>
       </c>
       <c r="I58" t="n">
-        <v>1.3</v>
+        <v>0.4</v>
       </c>
       <c r="J58" t="n">
         <v>0</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Юнусабадский район</t>
+          <t>Бектемирский район</t>
         </is>
       </c>
       <c r="L58" t="n">
-        <v>2632</v>
+        <v>10644</v>
       </c>
       <c r="M58" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N58" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O58" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q58" t="n">
         <v>0.5</v>
@@ -5859,13 +5859,13 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>139.7</v>
+        <v>60.2</v>
       </c>
       <c r="U58" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V58" t="n">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="W58" t="inlineStr">
         <is>
@@ -5879,7 +5879,7 @@
       </c>
       <c r="Y58" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.390081,69.264024</t>
+          <t>https://www.google.com/maps?q=41.254507,69.378627</t>
         </is>
       </c>
     </row>
@@ -5896,51 +5896,51 @@
         <v>68</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>41.254507</v>
+        <v>41.390081</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>69.37862699999999</v>
+        <v>69.26402400000001</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>41.254507, 69.378627</t>
+          <t>41.390081, 69.264024</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Сувсоз-2 (Водник)</t>
+          <t>Дустамабад</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>махалля</t>
+          <t>посёлок</t>
         </is>
       </c>
       <c r="I59" t="n">
-        <v>0.4</v>
+        <v>1.3</v>
       </c>
       <c r="J59" t="n">
         <v>0</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Бектемирский район</t>
+          <t>Юнусабадский район</t>
         </is>
       </c>
       <c r="L59" t="n">
-        <v>10644</v>
+        <v>2632</v>
       </c>
       <c r="M59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N59" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O59" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q59" t="n">
         <v>0.5</v>
@@ -5952,13 +5952,13 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>60.2</v>
+        <v>139.7</v>
       </c>
       <c r="U59" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V59" t="n">
-        <v>1500</v>
+        <v>500</v>
       </c>
       <c r="W59" t="inlineStr">
         <is>
@@ -5972,7 +5972,7 @@
       </c>
       <c r="Y59" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.254507,69.378627</t>
+          <t>https://www.google.com/maps?q=41.390081,69.264024</t>
         </is>
       </c>
     </row>
@@ -6024,7 +6024,7 @@
         <v>6883</v>
       </c>
       <c r="M60" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N60" t="n">
         <v>14</v>
@@ -6117,7 +6117,7 @@
         <v>4317</v>
       </c>
       <c r="M61" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N61" t="n">
         <v>7</v>
@@ -6210,7 +6210,7 @@
         <v>4927</v>
       </c>
       <c r="M62" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N62" t="n">
         <v>17</v>
@@ -6394,7 +6394,7 @@
         <v>1929</v>
       </c>
       <c r="M64" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N64" t="n">
         <v>18</v>
@@ -6487,7 +6487,7 @@
         <v>3879</v>
       </c>
       <c r="M65" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N65" t="n">
         <v>18</v>
@@ -6580,7 +6580,7 @@
         <v>1950</v>
       </c>
       <c r="M66" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N66" t="n">
         <v>22</v>
@@ -6635,7 +6635,7 @@
         <v>13</v>
       </c>
       <c r="C67" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D67" s="2" t="n">
         <v>41.36099</v>
@@ -6673,7 +6673,7 @@
         <v>2226</v>
       </c>
       <c r="M67" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N67" t="n">
         <v>16</v>
@@ -6728,7 +6728,7 @@
         <v>10</v>
       </c>
       <c r="C68" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D68" s="2" t="n">
         <v>41.370609</v>
@@ -6766,7 +6766,7 @@
         <v>3110</v>
       </c>
       <c r="M68" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N68" t="n">
         <v>15</v>
@@ -6859,7 +6859,7 @@
         <v>3499</v>
       </c>
       <c r="M69" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N69" t="n">
         <v>15</v>
@@ -6911,7 +6911,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C70" t="n">
         <v>69</v>
@@ -6952,7 +6952,7 @@
         <v>1357</v>
       </c>
       <c r="M70" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N70" t="n">
         <v>5</v>
@@ -7045,7 +7045,7 @@
         <v>4778</v>
       </c>
       <c r="M71" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N71" t="n">
         <v>11</v>
@@ -7100,7 +7100,7 @@
         <v>28</v>
       </c>
       <c r="C72" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D72" s="2" t="n">
         <v>41.361522</v>
@@ -7138,7 +7138,7 @@
         <v>1892</v>
       </c>
       <c r="M72" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N72" t="n">
         <v>6</v>
@@ -7188,7 +7188,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C73" t="n">
         <v>76</v>
@@ -7738,10 +7738,10 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C79" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D79" s="2" t="n">
         <v>41.33418</v>
@@ -7779,7 +7779,7 @@
         <v>1727</v>
       </c>
       <c r="M79" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N79" t="n">
         <v>7</v>
@@ -7832,7 +7832,7 @@
         <v>40</v>
       </c>
       <c r="C80" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D80" s="2" t="n">
         <v>41.399172</v>
@@ -7922,10 +7922,10 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C81" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D81" s="2" t="n">
         <v>41.401398</v>
@@ -8056,7 +8056,7 @@
         <v>4623</v>
       </c>
       <c r="M82" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N82" t="n">
         <v>11</v>
@@ -8201,7 +8201,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C84" t="n">
         <v>75</v>
@@ -8478,7 +8478,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C87" t="n">
         <v>73</v>
@@ -8569,10 +8569,10 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C88" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D88" s="2" t="n">
         <v>41.380099</v>
@@ -8660,10 +8660,10 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C89" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D89" s="2" t="n">
         <v>41.378499</v>
@@ -8844,7 +8844,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C91" t="n">
         <v>69</v>
@@ -9119,7 +9119,7 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C94" t="n">
         <v>73</v>
@@ -9210,10 +9210,10 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C95" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D95" s="2" t="n">
         <v>41.425276</v>
@@ -9301,7 +9301,7 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C96" t="n">
         <v>76</v>
@@ -9392,25 +9392,25 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C97" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D97" s="2" t="n">
-        <v>41.412151</v>
+        <v>41.404809</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>69.177485</v>
+        <v>69.391277</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>41.412151, 69.177485</t>
+          <t>41.404809, 69.391277</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Сагбан</t>
+          <t>Уткир</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -9426,35 +9426,35 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>Ташкентский район</t>
+          <t>Кибрайский район</t>
         </is>
       </c>
       <c r="L97" t="n">
-        <v>2486</v>
+        <v>1919</v>
       </c>
       <c r="M97" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N97" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P97" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q97" t="n">
         <v>5</v>
       </c>
       <c r="R97" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S97" t="n">
-        <v>1519</v>
+        <v>1398</v>
       </c>
       <c r="T97" t="n">
-        <v>270.6</v>
+        <v>213.9</v>
       </c>
       <c r="U97" t="n">
         <v>0</v>
@@ -9467,12 +9467,12 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>3 из 3</t>
+          <t>2 из 3</t>
         </is>
       </c>
       <c r="Y97" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.412151,69.177485</t>
+          <t>https://www.google.com/maps?q=41.404809,69.391277</t>
         </is>
       </c>
     </row>
@@ -9489,19 +9489,19 @@
         <v>75</v>
       </c>
       <c r="D98" s="2" t="n">
-        <v>41.404809</v>
+        <v>41.412151</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>69.391277</v>
+        <v>69.177485</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>41.404809, 69.391277</t>
+          <t>41.412151, 69.177485</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Уткир</t>
+          <t>Сагбан</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -9517,35 +9517,35 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>Кибрайский район</t>
+          <t>Ташкентский район</t>
         </is>
       </c>
       <c r="L98" t="n">
-        <v>1919</v>
+        <v>2486</v>
       </c>
       <c r="M98" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N98" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P98" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q98" t="n">
         <v>5</v>
       </c>
       <c r="R98" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S98" t="n">
-        <v>1398</v>
+        <v>1519</v>
       </c>
       <c r="T98" t="n">
-        <v>213.9</v>
+        <v>270.6</v>
       </c>
       <c r="U98" t="n">
         <v>0</v>
@@ -9558,12 +9558,12 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2 из 3</t>
+          <t>3 из 3</t>
         </is>
       </c>
       <c r="Y98" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=41.404809,69.391277</t>
+          <t>https://www.google.com/maps?q=41.412151,69.177485</t>
         </is>
       </c>
     </row>
@@ -9665,7 +9665,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C100" t="n">
         <v>76</v>
@@ -9756,7 +9756,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C101" t="n">
         <v>73</v>
@@ -9847,7 +9847,7 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C102" t="n">
         <v>74</v>
@@ -10032,7 +10032,7 @@
         <v>9</v>
       </c>
       <c r="C104" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D104" s="2" t="n">
         <v>41.434386</v>
@@ -10123,7 +10123,7 @@
         <v>46</v>
       </c>
       <c r="C105" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D105" s="2" t="n">
         <v>41.451813</v>
@@ -10211,7 +10211,7 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C106" t="n">
         <v>76</v>
@@ -10302,7 +10302,7 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C107" t="n">
         <v>69</v>
@@ -10575,7 +10575,7 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C110" t="n">
         <v>75</v>
@@ -10666,7 +10666,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C111" t="n">
         <v>77</v>
@@ -10939,7 +10939,7 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C114" t="n">
         <v>77</v>
@@ -11303,7 +11303,7 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C118" t="n">
         <v>74</v>
@@ -11485,7 +11485,7 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C120" t="n">
         <v>69</v>
@@ -11579,7 +11579,7 @@
         <v>41</v>
       </c>
       <c r="C121" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D121" s="2" t="n">
         <v>41.570059</v>
@@ -12308,7 +12308,7 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C129" t="n">
         <v>56</v>
@@ -13582,7 +13582,7 @@
         </is>
       </c>
       <c r="B143" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C143" t="n">
         <v>59</v>
@@ -13675,7 +13675,7 @@
         </is>
       </c>
       <c r="B144" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C144" t="n">
         <v>54</v>
@@ -13862,7 +13862,7 @@
         <v>7</v>
       </c>
       <c r="C146" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D146" s="2" t="n">
         <v>40.836137</v>
@@ -14589,7 +14589,7 @@
         </is>
       </c>
       <c r="B154" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C154" t="n">
         <v>54</v>
@@ -14680,7 +14680,7 @@
         </is>
       </c>
       <c r="B155" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C155" t="n">
         <v>56</v>
@@ -15501,7 +15501,7 @@
         </is>
       </c>
       <c r="B164" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C164" t="n">
         <v>59</v>
@@ -16505,7 +16505,7 @@
         <v>28</v>
       </c>
       <c r="C175" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D175" s="2" t="n">
         <v>40.985763</v>
@@ -17233,7 +17233,7 @@
         <v>1</v>
       </c>
       <c r="C183" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D183" s="2" t="n">
         <v>40.252947</v>

</xml_diff>